<commit_message>
27 import now working with preview
</commit_message>
<xml_diff>
--- a/data/Boulders_Ticklist.xlsx
+++ b/data/Boulders_Ticklist.xlsx
@@ -981,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2703,6 +2703,126 @@
         <v>46174</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>claras nye boulder</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>6c+</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>9a+</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Aarhus</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Al Greene</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>45768</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Nisu</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>6c</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Tierra media Albarracín</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>45213</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Zanzibar</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>The PLATEAU - Bouldering</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>45122</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="4294967292" verticalDpi="4294967292"/>

</xml_diff>

<commit_message>
logbook can now be edited
</commit_message>
<xml_diff>
--- a/data/Boulders_Ticklist.xlsx
+++ b/data/Boulders_Ticklist.xlsx
@@ -981,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q50"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2706,120 +2706,85 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>claras nye boulder</t>
+          <t>Al Greene</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>6c+</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
           <t>6a</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>9a+</t>
+          <t>6a</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Aarhus</t>
+          <t>Kjugekull</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>46177</v>
+        <v>45768</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Al Greene</t>
+          <t>Nisu</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>6a</t>
+          <t>7a</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>6a</t>
+          <t>6c</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Kjugekull</t>
+          <t>Albarracín</t>
         </is>
       </c>
       <c r="F48" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>45768</v>
+        <v>45213</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Nisu</t>
+          <t>Zanzibar</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>7a</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
+          <t>7a+</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>6c</t>
+          <t>7a+</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Tierra media Albarracín</t>
+          <t>Rocklands</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>45213</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Zanzibar</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>7a+</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>7a+</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>The PLATEAU - Bouldering</t>
-        </is>
-      </c>
-      <c r="F50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="4" t="n">
         <v>45122</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added climber as variable, to differentiate between climbers data
</commit_message>
<xml_diff>
--- a/data/Boulders_Ticklist.xlsx
+++ b/data/Boulders_Ticklist.xlsx
@@ -981,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q49"/>
+  <dimension ref="A1:Q95"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1028,6 +1028,11 @@
           <t>Dato</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Climber</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2742,7 +2747,6 @@
           <t>7a</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>6c</t>
@@ -2788,6 +2792,1497 @@
         <v>45122</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TESTER</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>6b+</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Tokerud</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>46179</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>NEW CLIMBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sommartid</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>46167</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sickboy</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>46167</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Yoda</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>46166</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Brick 'ard</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>46165</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>The 4-layer man in the 2-layer version</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>46165</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Foucault, helt enkelt!</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>46117</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Häleri</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>46114</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Ilse - she wolf of SS</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>46113</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Super-ghetto</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>46113</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Träben</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>46110</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Sommarnatt</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>46110</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Babar</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>46110</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Gitanic</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Tierra media Albarracín</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>46033</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Duck</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>45918</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Lithium</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>7c+</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>45918</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Tare Baby</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Stem Bastensen</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>45864</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>King Fisher</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Trolldalstjønna a.k.a. Justad</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>45858</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Kristallo</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Magic Wood</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>45840</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Jack the chipper</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Magic Wood</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>45840</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Höhenrausch</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Magic Wood</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>45839</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Piranja</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>7c+</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>7c+</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Magic Wood</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>45833</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>The Kick</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Fruberget</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>45808</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Illusion</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Mommehål</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>45806</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Tvekampen</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>8a</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>8a</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Hultastenen</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>45702</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Colosseum sittstart</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>45700</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Rocketeer</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>45517</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Ineschakra</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Arrastradero Albarracín</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>45216</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Rammstein</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Arrastradero Albarracín</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="4" t="n">
+        <v>45216</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Linds långa linje</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>6b+</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>6b+</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>45206</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Pinotage</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>SASSIES - Bouldering</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>45129</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Rhino</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>THE RHINO - Bouldering</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>45121</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Weichei</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>7c+</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>7c+</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>The PLATEAU - Bouldering</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="4" t="n">
+        <v>45118</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Hellfire</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>7c+</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>7c+</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ROADKILL CAFE - Bouldering &amp; Tradclimbing</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>45112</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Le Carnage</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Bas Cuvier</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="4" t="n">
+        <v>45012</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Den gamle och havet</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Hönö</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="4" t="n">
+        <v>44860</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Intermezzo</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>7c</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Magic Wood</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="4" t="n">
+        <v>44781</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Björntjänst sittstart</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>44665</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Colosseum</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>6c+</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>6c</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="4" t="n">
+        <v>44640</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Våroffer</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>7b</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="4" t="n">
+        <v>44640</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Rockstar</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="4" t="n">
+        <v>44639</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>The Office</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>7b+</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Björnblocket</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="4" t="n">
+        <v>44400</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Fina areten sittstart</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="4" t="n">
+        <v>44296</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Fina areten</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>7a</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="4" t="n">
+        <v>43569</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Ghetto</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>7a+</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Kjugekull</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" s="4" t="n">
+        <v>43569</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Magnushan</t>
+        </is>
+      </c>
+    </row>
+    <row r="95"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="4294967292" verticalDpi="4294967292"/>

</xml_diff>